<commit_message>
feat(ui): 整合 UI 自动化并兼容复用本机 Google Chrome
项目分型 kind=api|ui：api 走 Excel、ui 走 JSON，执行/报告/权限/环境按 file 全复用。

core/ui_runner：自带 Chromium 缺失时自动回退本机 Google Chrome（channel=chrome/beta），无需联网下载内核；截图默认落盘且 allure 存在时同时作附件，报告页 UI 步骤 Tab 可回指取图。

新增 ui_case_store + /api/ui-cases（CRUD/校验/查重/迁移/变量候选）与 12 动作字典；前端 CasesView 双形态 + UiCasesView/UiStepEditor + ReportView UI 步骤 Tab。

验证：unit_tests 27 全绿（http 服务 fixture 覆盖 cookie 提取），smoke_ui 端到端 35/0，smoke_full/authz/scripts/api_defs 44/79/62/117 全绿，前端 build 通过。
</commit_message>
<xml_diff>
--- a/data/api_cases.xlsx
+++ b/data/api_cases.xlsx
@@ -1067,7 +1067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N48"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3102,7 +3102,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ai_music_list_001</t>
+          <t>ai_task_del_001</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3112,12 +3112,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>模板音乐列表接口</t>
+          <t>音频任务删除接口</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>冒烟-正常入参</t>
+          <t>正常入参（需失败任务ID，暂不执行）</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3127,7 +3127,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3137,7 +3137,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>/ai/api/audio/recommend/music/list</t>
+          <t>/ai/api/audio/audiocreation/task/delete</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3147,19 +3147,19 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>{"userId": "{{user_id}}", "channelId": "10030113270", "pageCursor": null, "pageSize": 10}</t>
+          <t>{"channelId": "10030113270", "userId": "{{user_id}}", "taskIds": ["{{fail_task_id}}"]}</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>[["eq", "status_code", 200], ["not_null", "$.data"]]</t>
+          <t>[["eq", "status_code", 200], ["eq", "$.code", "0000"]]</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ai_music_list_002</t>
+          <t>ai_task_del_002</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3169,12 +3169,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>模板音乐列表接口</t>
+          <t>音频任务删除接口</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>userId不传</t>
+          <t>taskIds不传</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>/ai/api/audio/recommend/music/list</t>
+          <t>/ai/api/audio/audiocreation/task/delete</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3204,19 +3204,19 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>{"channelId": "10030113270", "pageCursor": null, "pageSize": 10}</t>
+          <t>{"channelId": "10030113270", "userId": "{{user_id}}"}</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>[["eq", "status_code", 200], ["not_null", "$.data"]]</t>
+          <t>[["eq", "status_code", 200], ["neq", "$.code", "0000"]]</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ai_music_list_003</t>
+          <t>ai_task_del_003</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3226,12 +3226,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>模板音乐列表接口</t>
+          <t>音频任务删除接口</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>channelId不传</t>
+          <t>taskIds传不存在的ID</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>/ai/api/audio/recommend/music/list</t>
+          <t>/ai/api/audio/audiocreation/task/delete</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3261,19 +3261,19 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>{"userId": "{{user_id}}", "pageCursor": null, "pageSize": 10}</t>
+          <t>{"channelId": "10030113270", "userId": "{{user_id}}", "taskIds": ["nonexist_99999"]}</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>[["eq", "status_code", 200], ["neq", "$.code", "0000"]]</t>
+          <t>[["eq", "status_code", 200]]</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ai_music_list_004</t>
+          <t>ai_task_del_004</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3283,12 +3283,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>模板音乐列表接口</t>
+          <t>音频任务删除接口</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>pageCursor不传</t>
+          <t>channelId不传</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3298,7 +3298,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3308,7 +3308,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>/ai/api/audio/recommend/music/list</t>
+          <t>/ai/api/audio/audiocreation/task/delete</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3318,580 +3318,10 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>{"userId": "{{user_id}}", "channelId": "10030113270", "pageSize": 10}</t>
+          <t>{"userId": "{{user_id}}", "taskIds": ["fake_id"]}</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
-        <is>
-          <t>[["eq", "status_code", 200], ["not_null", "$.data"]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>ai_music_list_005</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>一键成片·AI音频</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>模板音乐列表接口</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>pageSize不传</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>/ai/api/audio/recommend/music/list</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>{"Authorization": "{{token}}", "x-yun-api-version": "v1", "Content-Type": "application/json"}</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>{"userId": "{{user_id}}", "channelId": "10030113270", "pageCursor": null}</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>[["eq", "status_code", 200], ["not_null", "$.data"]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>ai_music_list_006</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>一键成片·AI音频</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>模板音乐列表接口</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>text不传</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>/ai/api/audio/recommend/music/list</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>{"Authorization": "{{token}}", "x-yun-api-version": "v1", "Content-Type": "application/json"}</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>{"userId": "{{user_id}}", "channelId": "10030113270", "pageCursor": null, "pageSize": 10}</t>
-        </is>
-      </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>[["eq", "status_code", 200], ["not_null", "$.data"]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>ai_music_list_007</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>一键成片·AI音频</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>模板音乐列表接口</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>text指定模板</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>/ai/api/audio/recommend/music/list</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>{"Authorization": "{{token}}", "x-yun-api-version": "v1", "Content-Type": "application/json"}</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>{"userId": "{{user_id}}", "channelId": "10030113270", "pageCursor": null, "pageSize": 10, "text": "轻快"}</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>[["eq", "status_code", 200], ["not_null", "$.data"]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>ai_config_get_001</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>一键成片·AI音频</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>查询模型与token计算公式接口</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>冒烟-正常入参</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>/ai/api/audio/audiocreation/config/get</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>{"Authorization": "{{token}}", "x-yun-api-version": "v1", "Content-Type": "application/json"}</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>{"channelId": "10030113270", "userId": "{{user_id}}"}</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>[["eq", "status_code", 200], ["not_null", "$.data"]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>ai_config_get_002</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>一键成片·AI音频</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>查询模型与token计算公式接口</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>channelId不传</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>/ai/api/audio/audiocreation/config/get</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>{"Authorization": "{{token}}", "x-yun-api-version": "v1", "Content-Type": "application/json"}</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>{"userId": "{{user_id}}"}</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>[["eq", "status_code", 200], ["neq", "$.code", "0000"]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>ai_config_get_003</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>一键成片·AI音频</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>查询模型与token计算公式接口</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>userId不传（实际可选）</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>/ai/api/audio/audiocreation/config/get</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>{"Authorization": "{{token}}", "x-yun-api-version": "v1", "Content-Type": "application/json"}</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>{"channelId": "10030113270"}</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>[["eq", "status_code", 200], ["not_null", "$.data"]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>ai_task_del_001</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>一键成片·AI音频</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>音频任务删除接口</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>正常入参（需失败任务ID，暂不执行）</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>/ai/api/audio/audiocreation/task/delete</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>{"Authorization": "{{token}}", "x-yun-api-version": "v1", "Content-Type": "application/json"}</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>{"channelId": "10030113270", "userId": "{{user_id}}", "taskIds": ["{{fail_task_id}}"]}</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>[["eq", "status_code", 200], ["eq", "$.code", "0000"]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>ai_task_del_002</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>一键成片·AI音频</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>音频任务删除接口</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>taskIds不传</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>/ai/api/audio/audiocreation/task/delete</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>{"Authorization": "{{token}}", "x-yun-api-version": "v1", "Content-Type": "application/json"}</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>{"channelId": "10030113270", "userId": "{{user_id}}"}</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>[["eq", "status_code", 200], ["neq", "$.code", "0000"]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>ai_task_del_003</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>一键成片·AI音频</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>音频任务删除接口</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>taskIds传不存在的ID</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>/ai/api/audio/audiocreation/task/delete</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>{"Authorization": "{{token}}", "x-yun-api-version": "v1", "Content-Type": "application/json"}</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>{"channelId": "10030113270", "userId": "{{user_id}}", "taskIds": ["nonexist_99999"]}</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>[["eq", "status_code", 200]]</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>ai_task_del_004</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>一键成片·AI音频</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>音频任务删除接口</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>channelId不传</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>/ai/api/audio/audiocreation/task/delete</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>{"Authorization": "{{token}}", "x-yun-api-version": "v1", "Content-Type": "application/json"}</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>{"userId": "{{user_id}}", "taskIds": ["fake_id"]}</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
         <is>
           <t>[["eq", "status_code", 200], ["neq", "$.code", "0000"]]</t>
         </is>

</xml_diff>